<commit_message>
Update 30-day content plan to the agreed calendar
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QodmTPnHVXWLRihnTm3bVa
</commit_message>
<xml_diff>
--- a/kanal/kontent-plan-30-dney.xlsx
+++ b/kanal/kontent-plan-30-dney.xlsx
@@ -38,7 +38,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00DDE7F5"/>
+        <fgColor rgb="00EFEAFF"/>
       </patternFill>
     </fill>
   </fills>
@@ -427,16 +427,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
-    <col width="32" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
-    <col width="36" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="2" max="2"/>
+    <col width="38" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="34" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -447,32 +445,22 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>День недели</t>
+          <t>Публикация</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Рубрика</t>
+          <t>Материал</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Формат</t>
+          <t>Готовый текст</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Цель</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Заголовок-хук</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>CTA</t>
+          <t>Призыв</t>
         </is>
       </c>
     </row>
@@ -484,698 +472,346 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Пн</t>
+          <t>Сколько часов уходит на обслуживание переписки</t>
         </is>
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>#с_чего_начать + #боль</t>
+          <t>Текст + закреп</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Закреп + пост</t>
+          <t>Пост 1</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Объяснить, куда пришли; узнавание боли</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="inlineStr">
-        <is>
-          <t>Сколько часов в неделю вы отвечаете «а где мой заказ?»</t>
-        </is>
-      </c>
-      <c r="G2" s="2" t="inlineStr">
-        <is>
-          <t>Напишите число часов в комментариях</t>
+          <t>Число часов в комментариях</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>3</t>
         </is>
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>Вт</t>
+          <t>Где теряется заказ в комментариях и личке</t>
         </is>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>#демо</t>
+          <t>Текст, разбор процесса</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Сторис (stories-1 бронь)</t>
+          <t>Написать</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Первое касание с продуктом</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Клиент бронирует сам — вы не переписываетесь</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Ссылка-стикер на демо-бота</t>
+          <t>Как принимаете заказы вы?</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>5</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>Ср</t>
+          <t>Как выглядит заказ через «Кнопку»</t>
         </is>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>#разбор</t>
+          <t>Готовое минутное видео</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Пост</t>
+          <t>Пост 3</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Польза без покупки, сохранения</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="inlineStr">
-        <is>
-          <t>Наценка 20 % превращается в 6 %: где теряется маржа посредника</t>
-        </is>
-      </c>
-      <c r="G4" s="2" t="inlineStr">
-        <is>
-          <t>Пришлите свои цифры — посчитаю</t>
+          <t>Демо-бот</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>Чт</t>
+          <t>Скрин оплаты — ещё не оплата</t>
         </is>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>#демо</t>
+          <t>Текст + опрос</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>Сторис (stories-2 оплата)</t>
+          <t>Пост 4</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Касание с продуктом</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="inlineStr">
-        <is>
-          <t>«Скинула скрин» — и вы час ищете перевод</t>
-        </is>
-      </c>
-      <c r="G5" s="2" t="inlineStr">
-        <is>
-          <t>Демо-бот</t>
+          <t>Опрос</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>10</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Пт</t>
+          <t>Какая работа повторяется чаще всего</t>
         </is>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>#демо</t>
+          <t>Опрос</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>Видео ≤ 60 с</t>
+          <t>Пост 5</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Показать вместо обещаний</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>Заказ глазами вашего клиента: 60 секунд</t>
-        </is>
-      </c>
-      <c r="G6" s="2" t="inlineStr">
-        <is>
-          <t>Попробовать демо-бота самому</t>
+          <t>Ответ в опросе</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>8</t>
+          <t>12</t>
         </is>
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Пн</t>
+          <t>«Где мой заказ?» — что можно показать клиенту без переписки</t>
         </is>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>#боль</t>
+          <t>Готовый ролик про статусы</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Пост</t>
+          <t>Написать подпись</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Цена потери в деньгах</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>Скрин оплаты — ещё не оплата</t>
-        </is>
-      </c>
-      <c r="G7" s="2" t="inlineStr">
-        <is>
-          <t>Опрос: было ли у вас такое?</t>
+          <t>Демо-бот</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>9</t>
+          <t>15</t>
         </is>
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Вт</t>
+          <t>По какому курсу вы считаете выкуп?</t>
         </is>
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>#демо</t>
+          <t>Текст, калькулятор и конвертации</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
-          <t>Сторис (stories-3 статусы)</t>
+          <t>Пост 2 (новый)</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Касание</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>Клиент сам видит, что заказ едет</t>
-        </is>
-      </c>
-      <c r="G8" s="2" t="inlineStr">
-        <is>
-          <t>Демо-бот</t>
+          <t>Пришлите свою схему — разберу</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>17</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Ср</t>
+          <t>Обзор возможностей «Кнопки»</t>
         </is>
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>#вопрос</t>
+          <t>Готовые 10 карточек альбомом</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Опрос</t>
+          <t>Пост 6</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Сегментация аудитории, вовлечение</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>Где вы сейчас ведёте заказы?</t>
-        </is>
-      </c>
-      <c r="G9" s="2" t="inlineStr">
-        <is>
-          <t>Ответить в опросе</t>
+          <t>Демо + условия в закрепе</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>19</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>Чт</t>
+          <t>Кейс № 1: один процесс до и после</t>
         </is>
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>#демо</t>
+          <t>Только подтверждённые факты, иначе перенос</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>Сторис (stories-4 защита)</t>
+          <t>Пост 9</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Касание</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>Как не нарваться на «покупателя-призрака»</t>
-        </is>
-      </c>
-      <c r="G10" s="2" t="inlineStr">
-        <is>
-          <t>Демо-бот</t>
+          <t>Пришлите, как у вас — разберу</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>12</t>
+          <t>22</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>Пт</t>
+          <t>Коллективный выкуп: что повторяется у организатора</t>
         </is>
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>#демо</t>
+          <t>Разбор + сторис про бронь</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>Карусель 10 карточек</t>
+          <t>Пост 7</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Полная картина продукта</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>Что умеет «Кнопка» — за 10 карточек</t>
-        </is>
-      </c>
-      <c r="G11" s="2" t="inlineStr">
-        <is>
-          <t>Демо + тарифы в закрепе</t>
+          <t>Пришлите, как у вас — разберу</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>15</t>
+          <t>24</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Пн</t>
+          <t>Вопросы о работе и подключении</t>
         </is>
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>#разбор</t>
+          <t>Кружок или короткое видео</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>Пост</t>
+          <t>Только реальные вопросы</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Польза + переход к разбору</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>Сбор на 30 человек: где теряются деньги и вечера</t>
-        </is>
-      </c>
-      <c r="G12" s="2" t="inlineStr">
-        <is>
-          <t>Анкета на бесплатный разбор</t>
+          <t>Задать следующий вопрос</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>16</t>
+          <t>26</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Вт</t>
+          <t>Кейс № 2 или разбор: бронь без предоплаты</t>
         </is>
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>#демо</t>
+          <t>Текст</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Сторис (stories-5 задачи)</t>
+          <t>Кейс по шаблону поста 9, иначе Пост 10</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Касание</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>Ничего не забыть: выкуп, отправка, доплата</t>
-        </is>
-      </c>
-      <c r="G13" s="2" t="inlineStr">
-        <is>
-          <t>Демо-бот</t>
+          <t>Демо брони</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>17</t>
+          <t>29</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Ср</t>
+          <t>Что автоматизировать первым в небольшом канале</t>
         </is>
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>#закулисье</t>
+          <t>Текст</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Пост</t>
+          <t>Написать</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Снятие риска по цене</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>Почему я беру процент, а не фикс</t>
-        </is>
-      </c>
-      <c r="G14" s="2" t="inlineStr">
-        <is>
-          <t>Вопросы в личку</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>18</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Чт</t>
-        </is>
-      </c>
-      <c r="C15" s="2" t="inlineStr">
-        <is>
-          <t>#демо</t>
-        </is>
-      </c>
-      <c r="D15" s="2" t="inlineStr">
-        <is>
-          <t>Сторис (stories-6 конкурсы)</t>
-        </is>
-      </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>Касание</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>Конкурс без таблиц и ручного подсчёта</t>
-        </is>
-      </c>
-      <c r="G15" s="2" t="inlineStr">
-        <is>
-          <t>Демо-бот</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="inlineStr">
-        <is>
-          <t>19</t>
-        </is>
-      </c>
-      <c r="B16" s="2" t="inlineStr">
-        <is>
-          <t>Пт</t>
-        </is>
-      </c>
-      <c r="C16" s="2" t="inlineStr">
-        <is>
-          <t>#кейс</t>
-        </is>
-      </c>
-      <c r="D16" s="2" t="inlineStr">
-        <is>
-          <t>Пост</t>
-        </is>
-      </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>Доказательство</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>Было: 3 часа в день в личке. Стало: … (цифры только с согласия)</t>
-        </is>
-      </c>
-      <c r="G16" s="2" t="inlineStr">
-        <is>
-          <t>Анкета на разбор</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="2" t="inlineStr">
-        <is>
-          <t>22</t>
-        </is>
-      </c>
-      <c r="B17" s="2" t="inlineStr">
-        <is>
-          <t>Пн</t>
-        </is>
-      </c>
-      <c r="C17" s="2" t="inlineStr">
-        <is>
-          <t>#разбор</t>
-        </is>
-      </c>
-      <c r="D17" s="2" t="inlineStr">
-        <is>
-          <t>Пост</t>
-        </is>
-      </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>Польза, сохранения</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>Бронь без предоплаты: 5 правил, чтобы не остаться с товаром</t>
-        </is>
-      </c>
-      <c r="G17" s="2" t="inlineStr">
-        <is>
-          <t>Демо брони</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>24</t>
-        </is>
-      </c>
-      <c r="B18" s="2" t="inlineStr">
-        <is>
-          <t>Ср</t>
-        </is>
-      </c>
-      <c r="C18" s="2" t="inlineStr">
-        <is>
-          <t>#вопрос</t>
-        </is>
-      </c>
-      <c r="D18" s="2" t="inlineStr">
-        <is>
-          <t>Кружок</t>
-        </is>
-      </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>Живой контакт, доверие</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>Отвечаю на 3 ваших вопроса за минуту</t>
-        </is>
-      </c>
-      <c r="G18" s="2" t="inlineStr">
-        <is>
-          <t>Задайте следующий вопрос в комментариях</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>26</t>
-        </is>
-      </c>
-      <c r="B19" s="2" t="inlineStr">
-        <is>
-          <t>Пт</t>
-        </is>
-      </c>
-      <c r="C19" s="2" t="inlineStr">
-        <is>
-          <t>#разбор</t>
-        </is>
-      </c>
-      <c r="D19" s="2" t="inlineStr">
-        <is>
-          <t>Пост-чек-лист</t>
-        </is>
-      </c>
-      <c r="E19" s="2" t="inlineStr">
-        <is>
-          <t>Польза, пересылки</t>
-        </is>
-      </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>Как проверить продавца перед оплатой: 7 пунктов</t>
-        </is>
-      </c>
-      <c r="G19" s="2" t="inlineStr">
-        <is>
-          <t>Переслать коллеге</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>29</t>
-        </is>
-      </c>
-      <c r="B20" s="2" t="inlineStr">
-        <is>
-          <t>Пн</t>
-        </is>
-      </c>
-      <c r="C20" s="2" t="inlineStr">
-        <is>
-          <t>#закулисье</t>
-        </is>
-      </c>
-      <c r="D20" s="2" t="inlineStr">
-        <is>
-          <t>Пост</t>
-        </is>
-      </c>
-      <c r="E20" s="2" t="inlineStr">
-        <is>
-          <t>Итоги + честная срочность</t>
-        </is>
-      </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>Месяц канала: что вы спросили и что я добавил</t>
-        </is>
-      </c>
-      <c r="G20" s="2" t="inlineStr">
-        <is>
-          <t>Разбор: осталось N мест в этом месяце</t>
+          <t>Приглашение на разбор</t>
         </is>
       </c>
     </row>

</xml_diff>